<commit_message>
Fix unit tests failing in master.
</commit_message>
<xml_diff>
--- a/client/tests/fixtures/mini-config/forms/app/pregnancy.xlsx
+++ b/client/tests/fixtures/mini-config/forms/app/pregnancy.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="60">
   <si>
     <t>type</t>
   </si>
@@ -64,6 +64,12 @@
   </si>
   <si>
     <t>end group</t>
+  </si>
+  <si>
+    <t>patient_sex</t>
+  </si>
+  <si>
+    <t>patient_id</t>
   </si>
   <si>
     <t>date</t>
@@ -563,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -729,45 +735,45 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s">
         <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G9" t="s">
         <v>9</v>
@@ -775,16 +781,16 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
         <v>9</v>
@@ -793,27 +799,27 @@
         <v>9</v>
       </c>
       <c r="G10" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E11" t="s">
         <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="G11" t="s">
         <v>9</v>
@@ -821,24 +827,70 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" t="s">
         <v>34</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D13" t="s">
         <v>35</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>36</v>
       </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" t="s">
         <v>9</v>
       </c>
     </row>
@@ -855,7 +907,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -869,27 +921,27 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
@@ -897,13 +949,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -911,30 +963,30 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -950,24 +1002,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>